<commit_message>
update country vs 903205de00501a3bb583cfa51d8f6e5e71f5132d
</commit_message>
<xml_diff>
--- a/ig/nr-add-vs-cs-to-id/StructureDefinition-fr-core-patient-nationality.xlsx
+++ b/ig/nr-add-vs-cs-to-id/StructureDefinition-fr-core-patient-nationality.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-01-29T12:36:14+00:00</t>
+    <t>2024-01-29T12:40:21+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -393,7 +393,7 @@
     <t>extensible</t>
   </si>
   <si>
-    <t>http://hl7.org/fhir/ValueSet/country</t>
+    <t>http://terminology.hl7.org/ValueSet/v3-Country</t>
   </si>
   <si>
     <t>Extension.value[x]</t>
@@ -778,7 +778,7 @@
     <col min="23" max="23" width="19.03515625" customWidth="true" bestFit="true"/>
     <col min="24" max="24" width="18.859375" customWidth="true" bestFit="true"/>
     <col min="25" max="25" width="21.57421875" customWidth="true" bestFit="true"/>
-    <col min="26" max="26" width="33.2421875" customWidth="true" bestFit="true"/>
+    <col min="26" max="26" width="44.3828125" customWidth="true" bestFit="true"/>
     <col min="27" max="27" width="6.34765625" customWidth="true" bestFit="true"/>
     <col min="28" max="28" width="22.71875" customWidth="true" bestFit="true"/>
     <col min="29" max="29" width="42.03515625" customWidth="true" bestFit="true"/>

</xml_diff>